<commit_message>
feat: link horasAnuales override to Funding Tracker + Engine Timeline
- When user overrides Hours/year, Funding Tracker and Engine Timeline
  recalculate using tachPerYear = horasAnuales / htRatio
- When live (no override), both use rateAnnual from server data
- MX module (Component Status) stays on live rate always
- Override indicator: ✏️ badge on Engine Timeline header and
  Funding Tracker subtitle when user projection is active
- Subtitle shows 'User projection' vs 'Live data' in Engine Timeline
</commit_message>
<xml_diff>
--- a/Analisis de costos/Analisis de costos.xlsx
+++ b/Analisis de costos/Analisis de costos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/santiagovaras/Documents/VScode/FlightLog AQI/Analisis de costos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D62872E2-39A4-7D47-B432-A1A2C12BC7EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{040B2712-E2DA-7A42-B6EB-FFADBDE7B539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{527A39D4-531F-5E46-BD05-60CC344C8C69}"/>
   </bookViews>
@@ -32608,21 +32608,21 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
+      <sheetData sheetId="10" refreshError="1"/>
+      <sheetData sheetId="11" refreshError="1"/>
+      <sheetData sheetId="12" refreshError="1"/>
+      <sheetData sheetId="13" refreshError="1"/>
+      <sheetData sheetId="14" refreshError="1"/>
+      <sheetData sheetId="15" refreshError="1"/>
       <sheetData sheetId="16">
         <row r="25">
           <cell r="J25">
@@ -32685,10 +32685,10 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
-      <sheetData sheetId="20"/>
+      <sheetData sheetId="17" refreshError="1"/>
+      <sheetData sheetId="18" refreshError="1"/>
+      <sheetData sheetId="19" refreshError="1"/>
+      <sheetData sheetId="20" refreshError="1"/>
       <sheetData sheetId="21">
         <row r="1739">
           <cell r="E1739">
@@ -32701,104 +32701,104 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="22"/>
-      <sheetData sheetId="23"/>
-      <sheetData sheetId="24"/>
-      <sheetData sheetId="25"/>
-      <sheetData sheetId="26"/>
-      <sheetData sheetId="27"/>
-      <sheetData sheetId="28"/>
-      <sheetData sheetId="29"/>
-      <sheetData sheetId="30"/>
-      <sheetData sheetId="31"/>
-      <sheetData sheetId="32"/>
-      <sheetData sheetId="33"/>
-      <sheetData sheetId="34"/>
-      <sheetData sheetId="35"/>
-      <sheetData sheetId="36"/>
-      <sheetData sheetId="37"/>
-      <sheetData sheetId="38"/>
-      <sheetData sheetId="39"/>
-      <sheetData sheetId="40"/>
-      <sheetData sheetId="41"/>
-      <sheetData sheetId="42"/>
-      <sheetData sheetId="43"/>
-      <sheetData sheetId="44"/>
-      <sheetData sheetId="45"/>
-      <sheetData sheetId="46"/>
-      <sheetData sheetId="47"/>
-      <sheetData sheetId="48"/>
-      <sheetData sheetId="49"/>
-      <sheetData sheetId="50"/>
-      <sheetData sheetId="51"/>
-      <sheetData sheetId="52"/>
-      <sheetData sheetId="53"/>
-      <sheetData sheetId="54"/>
-      <sheetData sheetId="55"/>
-      <sheetData sheetId="56"/>
-      <sheetData sheetId="57"/>
-      <sheetData sheetId="58"/>
-      <sheetData sheetId="59"/>
-      <sheetData sheetId="60"/>
-      <sheetData sheetId="61"/>
-      <sheetData sheetId="62"/>
-      <sheetData sheetId="63"/>
-      <sheetData sheetId="64"/>
-      <sheetData sheetId="65"/>
-      <sheetData sheetId="66"/>
-      <sheetData sheetId="67"/>
-      <sheetData sheetId="68"/>
-      <sheetData sheetId="69"/>
-      <sheetData sheetId="70"/>
-      <sheetData sheetId="71"/>
-      <sheetData sheetId="72"/>
-      <sheetData sheetId="73"/>
-      <sheetData sheetId="74"/>
-      <sheetData sheetId="75"/>
-      <sheetData sheetId="76"/>
-      <sheetData sheetId="77"/>
-      <sheetData sheetId="78"/>
-      <sheetData sheetId="79"/>
-      <sheetData sheetId="80"/>
-      <sheetData sheetId="81"/>
-      <sheetData sheetId="82"/>
-      <sheetData sheetId="83"/>
-      <sheetData sheetId="84"/>
-      <sheetData sheetId="85"/>
-      <sheetData sheetId="86"/>
-      <sheetData sheetId="87"/>
-      <sheetData sheetId="88"/>
-      <sheetData sheetId="89"/>
-      <sheetData sheetId="90"/>
-      <sheetData sheetId="91"/>
-      <sheetData sheetId="92"/>
-      <sheetData sheetId="93"/>
-      <sheetData sheetId="94"/>
-      <sheetData sheetId="95"/>
-      <sheetData sheetId="96"/>
-      <sheetData sheetId="97"/>
-      <sheetData sheetId="98"/>
-      <sheetData sheetId="99"/>
-      <sheetData sheetId="100"/>
-      <sheetData sheetId="101"/>
-      <sheetData sheetId="102"/>
-      <sheetData sheetId="103"/>
-      <sheetData sheetId="104"/>
-      <sheetData sheetId="105"/>
-      <sheetData sheetId="106"/>
-      <sheetData sheetId="107"/>
-      <sheetData sheetId="108"/>
-      <sheetData sheetId="109"/>
-      <sheetData sheetId="110"/>
-      <sheetData sheetId="111"/>
-      <sheetData sheetId="112"/>
-      <sheetData sheetId="113"/>
-      <sheetData sheetId="114"/>
-      <sheetData sheetId="115"/>
-      <sheetData sheetId="116"/>
-      <sheetData sheetId="117"/>
-      <sheetData sheetId="118"/>
-      <sheetData sheetId="119"/>
+      <sheetData sheetId="22" refreshError="1"/>
+      <sheetData sheetId="23" refreshError="1"/>
+      <sheetData sheetId="24" refreshError="1"/>
+      <sheetData sheetId="25" refreshError="1"/>
+      <sheetData sheetId="26" refreshError="1"/>
+      <sheetData sheetId="27" refreshError="1"/>
+      <sheetData sheetId="28" refreshError="1"/>
+      <sheetData sheetId="29" refreshError="1"/>
+      <sheetData sheetId="30" refreshError="1"/>
+      <sheetData sheetId="31" refreshError="1"/>
+      <sheetData sheetId="32" refreshError="1"/>
+      <sheetData sheetId="33" refreshError="1"/>
+      <sheetData sheetId="34" refreshError="1"/>
+      <sheetData sheetId="35" refreshError="1"/>
+      <sheetData sheetId="36" refreshError="1"/>
+      <sheetData sheetId="37" refreshError="1"/>
+      <sheetData sheetId="38" refreshError="1"/>
+      <sheetData sheetId="39" refreshError="1"/>
+      <sheetData sheetId="40" refreshError="1"/>
+      <sheetData sheetId="41" refreshError="1"/>
+      <sheetData sheetId="42" refreshError="1"/>
+      <sheetData sheetId="43" refreshError="1"/>
+      <sheetData sheetId="44" refreshError="1"/>
+      <sheetData sheetId="45" refreshError="1"/>
+      <sheetData sheetId="46" refreshError="1"/>
+      <sheetData sheetId="47" refreshError="1"/>
+      <sheetData sheetId="48" refreshError="1"/>
+      <sheetData sheetId="49" refreshError="1"/>
+      <sheetData sheetId="50" refreshError="1"/>
+      <sheetData sheetId="51" refreshError="1"/>
+      <sheetData sheetId="52" refreshError="1"/>
+      <sheetData sheetId="53" refreshError="1"/>
+      <sheetData sheetId="54" refreshError="1"/>
+      <sheetData sheetId="55" refreshError="1"/>
+      <sheetData sheetId="56" refreshError="1"/>
+      <sheetData sheetId="57" refreshError="1"/>
+      <sheetData sheetId="58" refreshError="1"/>
+      <sheetData sheetId="59" refreshError="1"/>
+      <sheetData sheetId="60" refreshError="1"/>
+      <sheetData sheetId="61" refreshError="1"/>
+      <sheetData sheetId="62" refreshError="1"/>
+      <sheetData sheetId="63" refreshError="1"/>
+      <sheetData sheetId="64" refreshError="1"/>
+      <sheetData sheetId="65" refreshError="1"/>
+      <sheetData sheetId="66" refreshError="1"/>
+      <sheetData sheetId="67" refreshError="1"/>
+      <sheetData sheetId="68" refreshError="1"/>
+      <sheetData sheetId="69" refreshError="1"/>
+      <sheetData sheetId="70" refreshError="1"/>
+      <sheetData sheetId="71" refreshError="1"/>
+      <sheetData sheetId="72" refreshError="1"/>
+      <sheetData sheetId="73" refreshError="1"/>
+      <sheetData sheetId="74" refreshError="1"/>
+      <sheetData sheetId="75" refreshError="1"/>
+      <sheetData sheetId="76" refreshError="1"/>
+      <sheetData sheetId="77" refreshError="1"/>
+      <sheetData sheetId="78" refreshError="1"/>
+      <sheetData sheetId="79" refreshError="1"/>
+      <sheetData sheetId="80" refreshError="1"/>
+      <sheetData sheetId="81" refreshError="1"/>
+      <sheetData sheetId="82" refreshError="1"/>
+      <sheetData sheetId="83" refreshError="1"/>
+      <sheetData sheetId="84" refreshError="1"/>
+      <sheetData sheetId="85" refreshError="1"/>
+      <sheetData sheetId="86" refreshError="1"/>
+      <sheetData sheetId="87" refreshError="1"/>
+      <sheetData sheetId="88" refreshError="1"/>
+      <sheetData sheetId="89" refreshError="1"/>
+      <sheetData sheetId="90" refreshError="1"/>
+      <sheetData sheetId="91" refreshError="1"/>
+      <sheetData sheetId="92" refreshError="1"/>
+      <sheetData sheetId="93" refreshError="1"/>
+      <sheetData sheetId="94" refreshError="1"/>
+      <sheetData sheetId="95" refreshError="1"/>
+      <sheetData sheetId="96" refreshError="1"/>
+      <sheetData sheetId="97" refreshError="1"/>
+      <sheetData sheetId="98" refreshError="1"/>
+      <sheetData sheetId="99" refreshError="1"/>
+      <sheetData sheetId="100" refreshError="1"/>
+      <sheetData sheetId="101" refreshError="1"/>
+      <sheetData sheetId="102" refreshError="1"/>
+      <sheetData sheetId="103" refreshError="1"/>
+      <sheetData sheetId="104" refreshError="1"/>
+      <sheetData sheetId="105" refreshError="1"/>
+      <sheetData sheetId="106" refreshError="1"/>
+      <sheetData sheetId="107" refreshError="1"/>
+      <sheetData sheetId="108" refreshError="1"/>
+      <sheetData sheetId="109" refreshError="1"/>
+      <sheetData sheetId="110" refreshError="1"/>
+      <sheetData sheetId="111" refreshError="1"/>
+      <sheetData sheetId="112" refreshError="1"/>
+      <sheetData sheetId="113" refreshError="1"/>
+      <sheetData sheetId="114" refreshError="1"/>
+      <sheetData sheetId="115" refreshError="1"/>
+      <sheetData sheetId="116" refreshError="1"/>
+      <sheetData sheetId="117" refreshError="1"/>
+      <sheetData sheetId="118" refreshError="1"/>
+      <sheetData sheetId="119" refreshError="1"/>
       <sheetData sheetId="120">
         <row r="1">
           <cell r="A1">
@@ -32826,7 +32826,7 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="121"/>
+      <sheetData sheetId="121" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>

</xml_diff>